<commit_message>
NUEVOS AJUSTES AL FORMATO
NUEVOS AJUSTES AL FORMATO
</commit_message>
<xml_diff>
--- a/assets/formatos-notas/formato_1_y_2_bgu.xlsx
+++ b/assets/formatos-notas/formato_1_y_2_bgu.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30131"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{656BE99A-8E43-42D9-A342-884AF7A01A56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6BC4EEB-B6BE-4366-8114-1B9DDAE30C31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -240,10 +240,10 @@
     <t>EMPRENDIMIENTO Y GESTIÓN</t>
   </si>
   <si>
-    <t>ACOMPAÑAMIENTO INTEGRAL EN EL AULA</t>
-  </si>
-  <si>
     <t>EVALUACIÓN COMPORTAMENTAL</t>
+  </si>
+  <si>
+    <t>CÍVICA Y ACOMPAÑAMIENTO INTEGRAL EN EL AULA</t>
   </si>
 </sst>
 </file>
@@ -692,7 +692,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AS18"/>
+  <dimension ref="A1:AS31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.21875" customWidth="1"/>
@@ -922,10 +922,10 @@
         <v>69</v>
       </c>
       <c r="O9" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="P9" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>71</v>
       </c>
       <c r="AN9" t="s">
         <v>64</v>
@@ -1099,15 +1099,281 @@
         <v>51</v>
       </c>
     </row>
-    <row r="17" spans="41:41" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A17" s="7"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="3"/>
       <c r="AO17" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="41:41" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A18" s="7"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
       <c r="AO18" t="s">
         <v>14</v>
       </c>
+    </row>
+    <row r="19" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A19" s="7"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="3"/>
+    </row>
+    <row r="20" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A20" s="7"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="3"/>
+      <c r="P20" s="3"/>
+    </row>
+    <row r="21" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A21" s="7"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+      <c r="P21" s="3"/>
+    </row>
+    <row r="22" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A22" s="7"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+      <c r="P22" s="3"/>
+    </row>
+    <row r="23" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A23" s="7"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+    </row>
+    <row r="24" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A24" s="7"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="3"/>
+    </row>
+    <row r="25" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A25" s="7"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+    </row>
+    <row r="26" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A26" s="7"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="P26" s="3"/>
+    </row>
+    <row r="27" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A27" s="7"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+    </row>
+    <row r="28" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A28" s="7"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+      <c r="P28" s="3"/>
+    </row>
+    <row r="29" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A29" s="7"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
+    </row>
+    <row r="30" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A30" s="7"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
+    </row>
+    <row r="31" spans="1:41" x14ac:dyDescent="0.3">
+      <c r="A31" s="7"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+      <c r="P31" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>